<commit_message>
Updated JPN_grids model - 2025-09-19 00:59
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33597F6A-7DB4-43D3-A75E-0B796240D426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F36AD2A4-5C9D-402C-9B21-38FE4B7FDD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -980,16 +980,130 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_023</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 23</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_017</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_019</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_030</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 30</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_003</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_029</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 29</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_031</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 31</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_020</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 20</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_028</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 28</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
+    <t>distr_solelc_spv_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_024</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 24</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_022</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 22</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_016</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_027</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 27</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_011</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_014</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_025</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 25</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_001</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 1</t>
   </si>
   <si>
     <t>distr_solelc_spv_018</t>
@@ -1010,12 +1124,6 @@
     <t>connecting solar to buses in cluster 7</t>
   </si>
   <si>
-    <t>distr_solelc_spv_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_012</t>
   </si>
   <si>
@@ -1028,78 +1136,6 @@
     <t>connecting solar to buses in cluster 15</t>
   </si>
   <si>
-    <t>distr_solelc_spv_022</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 22</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_016</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_027</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 27</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_017</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_019</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_030</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 30</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_003</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_029</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 29</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_031</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 31</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_024</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 24</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_023</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 23</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_010</t>
   </si>
   <si>
@@ -1118,42 +1154,6 @@
     <t>connecting solar to buses in cluster 9</t>
   </si>
   <si>
-    <t>distr_solelc_spv_011</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_014</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_025</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 25</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_020</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 20</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_001</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 1</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_021</t>
   </si>
   <si>
@@ -1178,9 +1178,63 @@
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_w216956620-500,e_JP219-500,e_JP132-500</t>
+  </si>
+  <si>
+    <t>e_w317416612-500,e_JP117-500,e_w242103481-500,e_w317511904-500,e_w242253537-500,e_JP137-500,e_JP135-500,e_JP120-500</t>
+  </si>
+  <si>
+    <t>e_w170974371-500,e_w171066843-500,e_w241828221-500,e_w87538349-500,e_w102958903-500,e_w241822623-500,e_w307942220-500,e_JP218-500</t>
+  </si>
+  <si>
+    <t>e_JP25-500,e_r17013811-500</t>
+  </si>
+  <si>
+    <t>e_w801582512-275,e_JP4-275,e_JP5-275,e_JP9-500,e_JP3-275,e_JP1-275</t>
+  </si>
+  <si>
+    <t>e_JP7-275,e_JP6-275,e_w179863079-275</t>
+  </si>
+  <si>
+    <t>e_JP21-500,e_w1030329139-500,e_w659138214-500,e_w106076988-500</t>
+  </si>
+  <si>
+    <t>e_w315618377-500,e_w256682313-500,e_JP74-500,e_JP25-500,e_w975217734-500,e_JP57-500,e_r17013811-500,e_w315662839-500,e_JP28-500</t>
+  </si>
+  <si>
+    <t>e_JP306-500</t>
+  </si>
+  <si>
     <t>e_w1030329139-500,e_w659138214-500,e_w253566674-500,e_JP19-500,e_w785319805-500,e_w106076988-500,e_w104173570-500,e_w901872431-500</t>
   </si>
   <si>
+    <t>e_w179863079-275</t>
+  </si>
+  <si>
+    <t>e_JP219-500,e_w150065045-500,e_w149843487-500,e_w145079972-500,e_w315461259-500,e_r2269992-500,e_JP132-500</t>
+  </si>
+  <si>
+    <t>e_JP296-500,e_w405626236-500,e_w201293312-500,e_w216778426-500,e_w1037299172-500,e_w172907196-500,e_w171066843-500,e_w722673849-500</t>
+  </si>
+  <si>
+    <t>e_w106076988-500,e_w174636874-500,e_JP10-500,e_w714627759-500</t>
+  </si>
+  <si>
+    <t>e_JP306-500,e_w215451416-500</t>
+  </si>
+  <si>
+    <t>e_JP248-500,e_w307942220-500,e_JP175-500,e_JP249-500,e_w291678103-500,e_w170605907-500,e_w1038584990-500,e_w109834508-500,e_w161727149-500,e_w421647841-500,e_JP116-500,e_w169031998-500,e_w170589736-500,e_JP156-500,e_JP122-500</t>
+  </si>
+  <si>
+    <t>e_w168727982-500,e_w132913106-500,e_w168839127-500,e_w105298089-500,e_w104391636-500,e_JP23-500</t>
+  </si>
+  <si>
+    <t>e_JP7-275,e_JP6-275</t>
+  </si>
+  <si>
+    <t>e_JP9-500,e_JP8-275,e_w1028554758-500</t>
+  </si>
+  <si>
     <t>e_w204258596-500,e_w242253500-500,e_w317416612-500,e_w193544791-500</t>
   </si>
   <si>
@@ -1190,94 +1244,82 @@
     <t>e_JP6-275</t>
   </si>
   <si>
-    <t>e_w179863079-275</t>
-  </si>
-  <si>
     <t>e_JP306-500,e_JP292-500,e_JP294-500,e_w172601929-500,e_w215451416-500,e_w216502300-500,e_w405626236-500,e_w172144358-500</t>
   </si>
   <si>
     <t>e_w216956620-500,e_w216953915-500</t>
   </si>
   <si>
-    <t>e_JP306-500</t>
-  </si>
-  <si>
-    <t>e_JP296-500,e_w405626236-500,e_w201293312-500,e_w216778426-500,e_w1037299172-500,e_w172907196-500,e_w171066843-500,e_w722673849-500</t>
-  </si>
-  <si>
-    <t>e_w106076988-500,e_w174636874-500,e_JP10-500,e_w714627759-500</t>
-  </si>
-  <si>
-    <t>e_w317416612-500,e_JP117-500,e_w242103481-500,e_w317511904-500,e_w242253537-500,e_JP137-500,e_JP135-500,e_JP120-500</t>
-  </si>
-  <si>
-    <t>e_w170974371-500,e_w171066843-500,e_w241828221-500,e_w87538349-500,e_w102958903-500,e_w241822623-500,e_w307942220-500,e_JP218-500</t>
-  </si>
-  <si>
-    <t>e_JP25-500,e_r17013811-500</t>
-  </si>
-  <si>
-    <t>e_w801582512-275,e_JP4-275,e_JP5-275,e_JP9-500,e_JP3-275,e_JP1-275</t>
-  </si>
-  <si>
-    <t>e_JP7-275,e_JP6-275,e_w179863079-275</t>
-  </si>
-  <si>
-    <t>e_JP21-500,e_w1030329139-500,e_w659138214-500,e_w106076988-500</t>
-  </si>
-  <si>
-    <t>e_w315618377-500,e_w256682313-500,e_JP74-500,e_JP25-500,e_w975217734-500,e_JP57-500,e_r17013811-500,e_w315662839-500,e_JP28-500</t>
-  </si>
-  <si>
-    <t>e_JP219-500,e_w150065045-500,e_w149843487-500,e_w145079972-500,e_w315461259-500,e_r2269992-500,e_JP132-500</t>
-  </si>
-  <si>
-    <t>e_w216956620-500,e_JP219-500,e_JP132-500</t>
-  </si>
-  <si>
     <t>e_JP269-500,e_w186510275-500,e_w185029969-500,e_w172601929-500,e_w187988970-500,e_w204258596-500</t>
   </si>
   <si>
     <t>e_w169031998-500,e_w170537514-500,e_JP96-500,e_w170247312-500,e_w170850727-500,e_w170366035-500,e_w116559939-500,e_w142662111-500,e_w209429410-500,e_w315662839-500,e_w210090094-500,e_w459476442-500,e_w209726348-500</t>
   </si>
   <si>
-    <t>e_JP7-275,e_JP6-275</t>
-  </si>
-  <si>
-    <t>e_JP306-500,e_w215451416-500</t>
-  </si>
-  <si>
-    <t>e_JP248-500,e_w307942220-500,e_JP175-500,e_JP249-500,e_w291678103-500,e_w170605907-500,e_w1038584990-500,e_w109834508-500,e_w161727149-500,e_w421647841-500,e_JP116-500,e_w169031998-500,e_w170589736-500,e_JP156-500,e_JP122-500</t>
-  </si>
-  <si>
-    <t>e_w168727982-500,e_w132913106-500,e_w168839127-500,e_w105298089-500,e_w104391636-500,e_JP23-500</t>
-  </si>
-  <si>
-    <t>e_JP9-500,e_JP8-275,e_w1028554758-500</t>
-  </si>
-  <si>
     <t>e_w106076988-500,e_w174636874-500,e_JP10-500</t>
   </si>
   <si>
     <t>e_w179863079-275,e_JP6-275</t>
   </si>
   <si>
+    <t>distr_wonelc_won_007</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_027</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 27</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_013</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_026</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 26</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_008</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 8</t>
   </si>
   <si>
-    <t>distr_wonelc_won_013</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_026</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 26</t>
+    <t>distr_wonelc_won_006</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_014</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_011</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_021</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 21</t>
   </si>
   <si>
     <t>distr_wonelc_won_028</t>
@@ -1292,6 +1334,18 @@
     <t>connecting wind onshore to buses in cluster 31</t>
   </si>
   <si>
+    <t>distr_wonelc_won_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_010</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 10</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_004</t>
   </si>
   <si>
@@ -1310,12 +1364,66 @@
     <t>connecting wind onshore to buses in cluster 23</t>
   </si>
   <si>
+    <t>distr_wonelc_won_024</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 24</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_019</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_018</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_005</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_029</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 29</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_016</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 16</t>
   </si>
   <si>
+    <t>distr_wonelc_won_009</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_022</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 22</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_025</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 25</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_030</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 30</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_017</t>
   </si>
   <si>
@@ -1334,118 +1442,40 @@
     <t>connecting wind onshore to buses in cluster 12</t>
   </si>
   <si>
-    <t>distr_wonelc_won_005</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_029</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 29</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_009</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_022</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 22</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_025</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 25</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_030</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 30</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_019</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_018</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_024</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 24</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_006</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_014</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_010</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 10</t>
-  </si>
-  <si>
     <t>distr_wonelc_won_015</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 15</t>
   </si>
   <si>
-    <t>distr_wonelc_won_007</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_027</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 27</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_011</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_021</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 21</t>
+    <t>elc_won_007</t>
+  </si>
+  <si>
+    <t>e_w169031998-500,e_w170537514-500,e_w170247312-500,e_w116559939-500</t>
+  </si>
+  <si>
+    <t>elc_won_027</t>
+  </si>
+  <si>
+    <t>e_w174636874-500,e_JP10-500,e_JP9-500,e_w714627759-500</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>e_JP219-500,e_JP132-500</t>
+  </si>
+  <si>
+    <t>elc_won_013</t>
+  </si>
+  <si>
+    <t>e_w149843487-500,e_w315461259-500,e_r2269992-500,e_JP132-500,e_w168727982-500,e_w132913106-500,e_w105298089-500</t>
+  </si>
+  <si>
+    <t>elc_won_026</t>
+  </si>
+  <si>
+    <t>e_w801582512-275,e_JP4-275,e_JP8-275,e_JP9-500,e_w1028554758-500,e_JP7-275</t>
   </si>
   <si>
     <t>elc_won_008</t>
@@ -1454,16 +1484,28 @@
     <t>e_w1038584990-500,e_w109834508-500,e_w161727149-500,e_w169031998-500,e_w170589736-500,e_JP156-500,e_w170537514-500,e_JP96-500,e_w170850727-500,e_w142662111-500</t>
   </si>
   <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>e_w149843487-500,e_w315461259-500,e_r2269992-500,e_JP132-500,e_w168727982-500,e_w132913106-500,e_w105298089-500</t>
-  </si>
-  <si>
-    <t>elc_won_026</t>
-  </si>
-  <si>
-    <t>e_w801582512-275,e_JP4-275,e_JP8-275,e_JP9-500,e_w1028554758-500,e_JP7-275</t>
+    <t>elc_won_006</t>
+  </si>
+  <si>
+    <t>e_JP294-500,e_w172601929-500,e_w215451416-500,e_w216502300-500,e_w405626236-500,e_w172144358-500,e_JP296-500</t>
+  </si>
+  <si>
+    <t>elc_won_014</t>
+  </si>
+  <si>
+    <t>e_w459476442-500,e_w150065045-500</t>
+  </si>
+  <si>
+    <t>elc_won_011</t>
+  </si>
+  <si>
+    <t>e_w242103481-500,e_w242253537-500,e_JP137-500,e_JP135-500,e_JP120-500,e_w421647841-500,e_JP116-500,e_w1029010255-500,e_JP122-500,e_w315618377-500</t>
+  </si>
+  <si>
+    <t>elc_won_021</t>
+  </si>
+  <si>
+    <t>e_w168839127-500,e_w104391636-500,e_w253566674-500,e_JP19-500,e_JP23-500,e_w104173570-500,e_w901872431-500,e_w106076988-500</t>
   </si>
   <si>
     <t>elc_won_028</t>
@@ -1472,6 +1514,18 @@
     <t>elc_won_031</t>
   </si>
   <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>e_JP306-500,e_w215451416-500,e_w216956620-500</t>
+  </si>
+  <si>
+    <t>elc_won_010</t>
+  </si>
+  <si>
+    <t>e_w216778426-500,e_w1037299172-500,e_w307942220-500,e_JP248-500,e_JP175-500,e_JP249-500,e_w291678103-500,e_w170605907-500</t>
+  </si>
+  <si>
     <t>elc_won_004</t>
   </si>
   <si>
@@ -1487,12 +1541,60 @@
     <t>e_JP21-500,e_w1030329139-500,e_w659138214-500</t>
   </si>
   <si>
+    <t>elc_won_024</t>
+  </si>
+  <si>
+    <t>e_w106076988-500,e_w785319805-500,e_w174636874-500</t>
+  </si>
+  <si>
+    <t>elc_won_019</t>
+  </si>
+  <si>
+    <t>e_JP292-500,e_JP269-500,e_w186510275-500,e_JP306-500,e_w185029969-500,e_w172601929-500,e_w187988970-500,e_w204258596-500</t>
+  </si>
+  <si>
+    <t>elc_won_018</t>
+  </si>
+  <si>
+    <t>e_w216956620-500,e_w216953915-500,e_JP296-500,e_w1037299172-500,e_w172907196-500,e_w722673849-500,e_JP249-500,e_w1038584990-500</t>
+  </si>
+  <si>
+    <t>elc_won_005</t>
+  </si>
+  <si>
+    <t>e_w201293312-500,e_w204258596-500,e_w242253500-500,e_w1037299172-500,e_w193544791-500,e_w317416612-500,e_w172907196-500,e_w170974371-500,e_w171066843-500,e_w241828221-500,e_w87538349-500,e_w102958903-500,e_w241822623-500,e_JP218-500</t>
+  </si>
+  <si>
+    <t>elc_won_029</t>
+  </si>
+  <si>
     <t>elc_won_016</t>
   </si>
   <si>
     <t>e_w204258596-500,e_w317416612-500,e_JP117-500,e_w317511904-500</t>
   </si>
   <si>
+    <t>elc_won_009</t>
+  </si>
+  <si>
+    <t>e_JP74-500,e_w975217734-500,e_JP57-500</t>
+  </si>
+  <si>
+    <t>elc_won_022</t>
+  </si>
+  <si>
+    <t>e_w315434358-500,e_w250540807-500,e_JP41-500,e_JP29-500,e_JP30-500</t>
+  </si>
+  <si>
+    <t>elc_won_025</t>
+  </si>
+  <si>
+    <t>e_w801582512-275,e_JP4-275,e_JP5-275,e_JP9-500,e_JP3-275,e_JP1-275,e_w179863079-275,e_JP7-275,e_JP6-275</t>
+  </si>
+  <si>
+    <t>elc_won_030</t>
+  </si>
+  <si>
     <t>elc_won_017</t>
   </si>
   <si>
@@ -1511,112 +1613,262 @@
     <t>e_w145079972-500,e_r15580570-500,e_w168839127-500</t>
   </si>
   <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>e_w201293312-500,e_w204258596-500,e_w242253500-500,e_w1037299172-500,e_w193544791-500,e_w317416612-500,e_w172907196-500,e_w170974371-500,e_w171066843-500,e_w241828221-500,e_w87538349-500,e_w102958903-500,e_w241822623-500,e_JP218-500</t>
-  </si>
-  <si>
-    <t>elc_won_029</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>e_JP74-500,e_w975217734-500,e_JP57-500</t>
-  </si>
-  <si>
-    <t>elc_won_022</t>
-  </si>
-  <si>
-    <t>e_w315434358-500,e_w250540807-500,e_JP41-500,e_JP29-500,e_JP30-500</t>
-  </si>
-  <si>
-    <t>elc_won_025</t>
-  </si>
-  <si>
-    <t>e_w801582512-275,e_JP4-275,e_JP5-275,e_JP9-500,e_JP3-275,e_JP1-275,e_w179863079-275,e_JP7-275,e_JP6-275</t>
-  </si>
-  <si>
-    <t>elc_won_030</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>e_JP292-500,e_JP269-500,e_w186510275-500,e_JP306-500,e_w185029969-500,e_w172601929-500,e_w187988970-500,e_w204258596-500</t>
-  </si>
-  <si>
-    <t>elc_won_018</t>
-  </si>
-  <si>
-    <t>e_w216956620-500,e_w216953915-500,e_JP296-500,e_w1037299172-500,e_w172907196-500,e_w722673849-500,e_JP249-500,e_w1038584990-500</t>
-  </si>
-  <si>
-    <t>elc_won_024</t>
-  </si>
-  <si>
-    <t>e_w106076988-500,e_w785319805-500,e_w174636874-500</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>e_JP294-500,e_w172601929-500,e_w215451416-500,e_w216502300-500,e_w405626236-500,e_w172144358-500,e_JP296-500</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>e_w459476442-500,e_w150065045-500</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>e_JP306-500,e_w215451416-500,e_w216956620-500</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>e_w216778426-500,e_w1037299172-500,e_w307942220-500,e_JP248-500,e_JP175-500,e_JP249-500,e_w291678103-500,e_w170605907-500</t>
-  </si>
-  <si>
     <t>elc_won_015</t>
   </si>
   <si>
     <t>e_w210090094-500,e_JP219-500,e_w150065045-500,e_w149843487-500,e_w315461259-500,e_JP132-500</t>
   </si>
   <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>e_w169031998-500,e_w170537514-500,e_w170247312-500,e_w116559939-500</t>
-  </si>
-  <si>
-    <t>elc_won_027</t>
-  </si>
-  <si>
-    <t>e_w174636874-500,e_JP10-500,e_JP9-500,e_w714627759-500</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>e_JP219-500,e_JP132-500</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>e_w242103481-500,e_w242253537-500,e_JP137-500,e_JP135-500,e_JP120-500,e_w421647841-500,e_JP116-500,e_w1029010255-500,e_JP122-500,e_w315618377-500</t>
-  </si>
-  <si>
-    <t>elc_won_021</t>
-  </si>
-  <si>
-    <t>e_w168839127-500,e_w104391636-500,e_w253566674-500,e_JP19-500,e_JP23-500,e_w104173570-500,e_w901872431-500,e_w106076988-500</t>
+    <t>distr_wofelc_wof_029</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 29</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_024</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 24</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_044</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 44</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_015</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_018</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_014</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_038</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 38</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_026</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 26</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_040</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 40</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_043</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 43</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_011</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_010</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_041</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 41</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_020</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 20</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_006</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_031</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 31</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_039</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 39</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_016</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_030</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 30</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_021</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 21</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_035</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 35</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_042</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 42</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_004</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_032</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 32</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_037</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 37</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_022</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 22</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_019</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_013</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_007</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_028</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 28</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_008</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_034</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 34</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_023</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 23</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_001</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_002</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_003</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_012</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_027</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 27</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_025</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 25</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_009</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_036</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 36</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_017</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 17</t>
   </si>
   <si>
     <t>distr_wofelc_wof_005</t>
@@ -1631,475 +1883,223 @@
     <t>connecting wind offshore to buses in cluster 33</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_040</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 40</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_043</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 43</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_026</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 26</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_028</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 28</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_008</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_034</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 34</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_019</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_007</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_004</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_032</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 32</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_037</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 37</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_022</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 22</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_013</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_001</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_002</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_003</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_012</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_027</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 27</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_025</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 25</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_014</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_038</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 38</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_030</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 30</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_021</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 21</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_035</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 35</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_042</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 42</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_009</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_036</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 36</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_017</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_011</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_010</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_041</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 41</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_020</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 20</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_006</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_031</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 31</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_039</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 39</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_016</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_029</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 29</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_024</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 24</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_044</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 44</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_015</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_018</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_023</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 23</t>
+    <t>elc_wof_029</t>
+  </si>
+  <si>
+    <t>e_w317416612-500,e_JP117-500</t>
+  </si>
+  <si>
+    <t>elc_wof_024</t>
+  </si>
+  <si>
+    <t>e_JP21-500,e_w174636874-500,e_w659138214-500,e_w106076988-500,e_JP10-500</t>
+  </si>
+  <si>
+    <t>elc_wof_044</t>
+  </si>
+  <si>
+    <t>e_w149843487-500,e_w315461259-500,e_JP132-500,e_w151379730-500,e_w168727982-500,e_w105298089-500</t>
+  </si>
+  <si>
+    <t>elc_wof_015</t>
+  </si>
+  <si>
+    <t>e_JP4-275,e_w179863079-275,e_JP7-275</t>
+  </si>
+  <si>
+    <t>elc_wof_018</t>
+  </si>
+  <si>
+    <t>elc_wof_014</t>
+  </si>
+  <si>
+    <t>e_JP269-500,e_JP292-500,e_w186510275-500</t>
+  </si>
+  <si>
+    <t>elc_wof_038</t>
+  </si>
+  <si>
+    <t>e_JP219-500</t>
+  </si>
+  <si>
+    <t>elc_wof_026</t>
+  </si>
+  <si>
+    <t>e_JP25-500,e_w256682313-500,e_r17013811-500</t>
+  </si>
+  <si>
+    <t>elc_wof_040</t>
+  </si>
+  <si>
+    <t>e_w170247312-500,e_JP219-500</t>
+  </si>
+  <si>
+    <t>elc_wof_043</t>
+  </si>
+  <si>
+    <t>e_w105298089-500,e_JP23-500,e_w104173570-500</t>
+  </si>
+  <si>
+    <t>elc_wof_011</t>
+  </si>
+  <si>
+    <t>e_JP306-500,e_w216956620-500,e_w215451416-500</t>
+  </si>
+  <si>
+    <t>elc_wof_010</t>
+  </si>
+  <si>
+    <t>e_w216778426-500,e_w1037299172-500,e_w722673849-500,e_w1037516198-500,e_w291678103-500,e_w1038584990-500</t>
+  </si>
+  <si>
+    <t>elc_wof_041</t>
+  </si>
+  <si>
+    <t>e_w156208858-500,e_w901872431-500,e_w104173570-500,e_w106076988-500</t>
+  </si>
+  <si>
+    <t>elc_wof_020</t>
+  </si>
+  <si>
+    <t>e_JP6-275,e_w179863079-275</t>
+  </si>
+  <si>
+    <t>elc_wof_006</t>
+  </si>
+  <si>
+    <t>elc_wof_031</t>
+  </si>
+  <si>
+    <t>e_JP121-500,e_w1029010255-500,e_w315618377-500,e_w256682313-500</t>
+  </si>
+  <si>
+    <t>elc_wof_039</t>
+  </si>
+  <si>
+    <t>e_JP219-500,e_w149843487-500,e_JP132-500,e_w315461259-500</t>
+  </si>
+  <si>
+    <t>elc_wof_016</t>
+  </si>
+  <si>
+    <t>e_w1028554758-500,e_JP9-500,e_JP5-275,e_JP7-275,e_w714627759-500</t>
+  </si>
+  <si>
+    <t>elc_wof_030</t>
+  </si>
+  <si>
+    <t>e_JP117-500</t>
+  </si>
+  <si>
+    <t>elc_wof_021</t>
+  </si>
+  <si>
+    <t>e_JP4-275,e_JP1-275,e_w179863079-275</t>
+  </si>
+  <si>
+    <t>elc_wof_035</t>
+  </si>
+  <si>
+    <t>elc_wof_042</t>
+  </si>
+  <si>
+    <t>e_w156208858-500,e_w901872431-500,e_w106076988-500,e_w174636874-500</t>
+  </si>
+  <si>
+    <t>elc_wof_004</t>
+  </si>
+  <si>
+    <t>elc_wof_032</t>
+  </si>
+  <si>
+    <t>e_w317511904-500,e_JP117-500,e_w242103481-500,e_w242253537-500,e_JP137-500,e_JP120-500,e_JP25-500</t>
+  </si>
+  <si>
+    <t>elc_wof_037</t>
+  </si>
+  <si>
+    <t>elc_wof_022</t>
+  </si>
+  <si>
+    <t>elc_wof_019</t>
+  </si>
+  <si>
+    <t>elc_wof_013</t>
+  </si>
+  <si>
+    <t>e_w186510275-500,e_w187988970-500,e_w204258596-500</t>
+  </si>
+  <si>
+    <t>elc_wof_007</t>
+  </si>
+  <si>
+    <t>elc_wof_028</t>
+  </si>
+  <si>
+    <t>e_w186510275-500,e_w204258596-500,e_w317416612-500</t>
+  </si>
+  <si>
+    <t>elc_wof_008</t>
+  </si>
+  <si>
+    <t>elc_wof_034</t>
+  </si>
+  <si>
+    <t>e_JP132-500,e_w105298089-500</t>
+  </si>
+  <si>
+    <t>elc_wof_023</t>
+  </si>
+  <si>
+    <t>elc_wof_001</t>
+  </si>
+  <si>
+    <t>elc_wof_002</t>
+  </si>
+  <si>
+    <t>elc_wof_003</t>
+  </si>
+  <si>
+    <t>elc_wof_012</t>
+  </si>
+  <si>
+    <t>e_JP292-500,e_JP269-500,e_JP306-500</t>
+  </si>
+  <si>
+    <t>elc_wof_027</t>
+  </si>
+  <si>
+    <t>e_JP25-500,e_JP21-500</t>
+  </si>
+  <si>
+    <t>elc_wof_025</t>
+  </si>
+  <si>
+    <t>e_r17013811-500,e_JP21-500</t>
+  </si>
+  <si>
+    <t>elc_wof_009</t>
+  </si>
+  <si>
+    <t>e_w1037299172-500,e_w172907196-500,e_w171066843-500,e_w722673849-500,e_w1037516198-500,e_JP249-500,e_w1038584990-500</t>
+  </si>
+  <si>
+    <t>elc_wof_036</t>
+  </si>
+  <si>
+    <t>e_w216956620-500,e_JP219-500</t>
+  </si>
+  <si>
+    <t>elc_wof_017</t>
+  </si>
+  <si>
+    <t>e_JP8-275,e_w801582512-275,e_JP9-500,e_JP10-500,e_w714627759-500</t>
   </si>
   <si>
     <t>elc_wof_005</t>
   </si>
   <si>
     <t>elc_wof_033</t>
-  </si>
-  <si>
-    <t>elc_wof_040</t>
-  </si>
-  <si>
-    <t>e_w170247312-500,e_JP219-500</t>
-  </si>
-  <si>
-    <t>elc_wof_043</t>
-  </si>
-  <si>
-    <t>e_w105298089-500,e_JP23-500,e_w104173570-500</t>
-  </si>
-  <si>
-    <t>elc_wof_026</t>
-  </si>
-  <si>
-    <t>e_JP25-500,e_w256682313-500,e_r17013811-500</t>
-  </si>
-  <si>
-    <t>elc_wof_028</t>
-  </si>
-  <si>
-    <t>e_w186510275-500,e_w204258596-500,e_w317416612-500</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>elc_wof_034</t>
-  </si>
-  <si>
-    <t>e_JP132-500,e_w105298089-500</t>
-  </si>
-  <si>
-    <t>elc_wof_019</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>elc_wof_004</t>
-  </si>
-  <si>
-    <t>elc_wof_032</t>
-  </si>
-  <si>
-    <t>e_w317511904-500,e_JP117-500,e_w242103481-500,e_w242253537-500,e_JP137-500,e_JP120-500,e_JP25-500</t>
-  </si>
-  <si>
-    <t>elc_wof_037</t>
-  </si>
-  <si>
-    <t>elc_wof_022</t>
-  </si>
-  <si>
-    <t>elc_wof_013</t>
-  </si>
-  <si>
-    <t>e_w186510275-500,e_w187988970-500,e_w204258596-500</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_012</t>
-  </si>
-  <si>
-    <t>e_JP292-500,e_JP269-500,e_JP306-500</t>
-  </si>
-  <si>
-    <t>elc_wof_027</t>
-  </si>
-  <si>
-    <t>e_JP25-500,e_JP21-500</t>
-  </si>
-  <si>
-    <t>elc_wof_025</t>
-  </si>
-  <si>
-    <t>e_r17013811-500,e_JP21-500</t>
-  </si>
-  <si>
-    <t>elc_wof_014</t>
-  </si>
-  <si>
-    <t>e_JP269-500,e_JP292-500,e_w186510275-500</t>
-  </si>
-  <si>
-    <t>elc_wof_038</t>
-  </si>
-  <si>
-    <t>e_JP219-500</t>
-  </si>
-  <si>
-    <t>elc_wof_030</t>
-  </si>
-  <si>
-    <t>e_JP117-500</t>
-  </si>
-  <si>
-    <t>elc_wof_021</t>
-  </si>
-  <si>
-    <t>e_JP4-275,e_JP1-275,e_w179863079-275</t>
-  </si>
-  <si>
-    <t>elc_wof_035</t>
-  </si>
-  <si>
-    <t>elc_wof_042</t>
-  </si>
-  <si>
-    <t>e_w156208858-500,e_w901872431-500,e_w106076988-500,e_w174636874-500</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>e_w1037299172-500,e_w172907196-500,e_w171066843-500,e_w722673849-500,e_w1037516198-500,e_JP249-500,e_w1038584990-500</t>
-  </si>
-  <si>
-    <t>elc_wof_036</t>
-  </si>
-  <si>
-    <t>e_w216956620-500,e_JP219-500</t>
-  </si>
-  <si>
-    <t>elc_wof_017</t>
-  </si>
-  <si>
-    <t>e_JP8-275,e_w801582512-275,e_JP9-500,e_JP10-500,e_w714627759-500</t>
-  </si>
-  <si>
-    <t>elc_wof_011</t>
-  </si>
-  <si>
-    <t>e_JP306-500,e_w216956620-500,e_w215451416-500</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
-  </si>
-  <si>
-    <t>e_w216778426-500,e_w1037299172-500,e_w722673849-500,e_w1037516198-500,e_w291678103-500,e_w1038584990-500</t>
-  </si>
-  <si>
-    <t>elc_wof_041</t>
-  </si>
-  <si>
-    <t>e_w156208858-500,e_w901872431-500,e_w104173570-500,e_w106076988-500</t>
-  </si>
-  <si>
-    <t>elc_wof_020</t>
-  </si>
-  <si>
-    <t>e_JP6-275,e_w179863079-275</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>elc_wof_031</t>
-  </si>
-  <si>
-    <t>e_JP121-500,e_w1029010255-500,e_w315618377-500,e_w256682313-500</t>
-  </si>
-  <si>
-    <t>elc_wof_039</t>
-  </si>
-  <si>
-    <t>e_JP219-500,e_w149843487-500,e_JP132-500,e_w315461259-500</t>
-  </si>
-  <si>
-    <t>elc_wof_016</t>
-  </si>
-  <si>
-    <t>e_w1028554758-500,e_JP9-500,e_JP5-275,e_JP7-275,e_w714627759-500</t>
-  </si>
-  <si>
-    <t>elc_wof_029</t>
-  </si>
-  <si>
-    <t>e_w317416612-500,e_JP117-500</t>
-  </si>
-  <si>
-    <t>elc_wof_024</t>
-  </si>
-  <si>
-    <t>e_JP21-500,e_w174636874-500,e_w659138214-500,e_w106076988-500,e_JP10-500</t>
-  </si>
-  <si>
-    <t>elc_wof_044</t>
-  </si>
-  <si>
-    <t>e_w149843487-500,e_w315461259-500,e_JP132-500,e_w151379730-500,e_w168727982-500,e_w105298089-500</t>
-  </si>
-  <si>
-    <t>elc_wof_015</t>
-  </si>
-  <si>
-    <t>e_JP4-275,e_w179863079-275,e_JP7-275</t>
-  </si>
-  <si>
-    <t>elc_wof_018</t>
-  </si>
-  <si>
-    <t>elc_wof_023</t>
   </si>
   <si>
     <t>e_won_001</t>
@@ -7576,7 +7576,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04E3DCEE-918C-4564-A09E-998D4F26F72E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7435C97D-E728-4F2F-880A-1A458C6B9EBC}">
   <dimension ref="B9:BD54"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7814,16 +7814,16 @@
         <v>283</v>
       </c>
       <c r="Y11" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="Z11" t="s">
         <v>349</v>
       </c>
       <c r="AA11">
-        <v>0.99798824264234642</v>
+        <v>0.9488788277802801</v>
       </c>
       <c r="AB11">
-        <v>36.882218223648351</v>
+        <v>937.22149069486488</v>
       </c>
       <c r="AD11" t="s">
         <v>282</v>
@@ -7856,10 +7856,10 @@
         <v>440</v>
       </c>
       <c r="AO11">
-        <v>0.99869874972548245</v>
+        <v>0.99710631799330929</v>
       </c>
       <c r="AP11">
-        <v>23.856255032822389</v>
+        <v>53.050836789329388</v>
       </c>
       <c r="AR11" t="s">
         <v>282</v>
@@ -7889,13 +7889,13 @@
         <v>584</v>
       </c>
       <c r="BB11" t="s">
-        <v>449</v>
+        <v>585</v>
       </c>
       <c r="BC11">
-        <v>0.95726256957223688</v>
+        <v>0.99490784156958001</v>
       </c>
       <c r="BD11">
-        <v>783.51955784232393</v>
+        <v>93.356237891033686</v>
       </c>
     </row>
     <row r="12" spans="2:56">
@@ -7960,16 +7960,16 @@
         <v>287</v>
       </c>
       <c r="Y12" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="Z12" t="s">
         <v>350</v>
       </c>
       <c r="AA12">
-        <v>0.99825665520226836</v>
+        <v>0.99809166649408687</v>
       </c>
       <c r="AB12">
-        <v>31.96132129174655</v>
+        <v>34.986114275074357</v>
       </c>
       <c r="AD12" t="s">
         <v>282</v>
@@ -8002,10 +8002,10 @@
         <v>442</v>
       </c>
       <c r="AO12">
-        <v>0.99863922747017897</v>
+        <v>0.99550555557680764</v>
       </c>
       <c r="AP12">
-        <v>24.947496380053089</v>
+        <v>82.398147758527074</v>
       </c>
       <c r="AR12" t="s">
         <v>282</v>
@@ -8032,16 +8032,16 @@
         <v>498</v>
       </c>
       <c r="BA12" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="BB12" t="s">
-        <v>491</v>
+        <v>587</v>
       </c>
       <c r="BC12">
-        <v>0.9437657388784082</v>
+        <v>0.99015836110796274</v>
       </c>
       <c r="BD12">
-        <v>1030.9614538958492</v>
+        <v>180.43004635401576</v>
       </c>
     </row>
     <row r="13" spans="2:56">
@@ -8106,16 +8106,16 @@
         <v>289</v>
       </c>
       <c r="Y13" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="Z13" t="s">
         <v>351</v>
       </c>
       <c r="AA13">
-        <v>0.99894650606645485</v>
+        <v>0.99850557699173803</v>
       </c>
       <c r="AB13">
-        <v>19.314055448326833</v>
+        <v>27.397755151469518</v>
       </c>
       <c r="AD13" t="s">
         <v>282</v>
@@ -8148,10 +8148,10 @@
         <v>444</v>
       </c>
       <c r="AO13">
-        <v>0.99582230548799566</v>
+        <v>0.93896180472603763</v>
       </c>
       <c r="AP13">
-        <v>76.591066053413869</v>
+        <v>1119.0335800226442</v>
       </c>
       <c r="AR13" t="s">
         <v>282</v>
@@ -8178,16 +8178,16 @@
         <v>500</v>
       </c>
       <c r="BA13" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="BB13" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="BC13">
-        <v>0.99681267676383467</v>
+        <v>0.99623532634854861</v>
       </c>
       <c r="BD13">
-        <v>58.434259329697142</v>
+        <v>69.01901694327529</v>
       </c>
     </row>
     <row r="14" spans="2:56">
@@ -8252,16 +8252,16 @@
         <v>291</v>
       </c>
       <c r="Y14" t="s">
-        <v>256</v>
+        <v>279</v>
       </c>
       <c r="Z14" t="s">
         <v>352</v>
       </c>
       <c r="AA14">
-        <v>0.98179245618315802</v>
+        <v>0.99621285878087551</v>
       </c>
       <c r="AB14">
-        <v>333.80496997543548</v>
+        <v>69.43092235061502</v>
       </c>
       <c r="AD14" t="s">
         <v>282</v>
@@ -8291,13 +8291,13 @@
         <v>445</v>
       </c>
       <c r="AN14" t="s">
-        <v>376</v>
+        <v>446</v>
       </c>
       <c r="AO14">
-        <v>0.99192535126433146</v>
+        <v>0.99863922747017897</v>
       </c>
       <c r="AP14">
-        <v>148.0352268205892</v>
+        <v>24.947496380053089</v>
       </c>
       <c r="AR14" t="s">
         <v>282</v>
@@ -8324,16 +8324,16 @@
         <v>502</v>
       </c>
       <c r="BA14" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="BB14" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="BC14">
-        <v>0.99602290686668338</v>
+        <v>0.9966173923071765</v>
       </c>
       <c r="BD14">
-        <v>72.91337411080552</v>
+        <v>62.014474368430825</v>
       </c>
     </row>
     <row r="15" spans="2:56">
@@ -8398,16 +8398,16 @@
         <v>293</v>
       </c>
       <c r="Y15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="Z15" t="s">
         <v>353</v>
       </c>
       <c r="AA15">
-        <v>0.99116451092312863</v>
+        <v>0.9975431479552237</v>
       </c>
       <c r="AB15">
-        <v>161.98396640930775</v>
+        <v>45.042287487565297</v>
       </c>
       <c r="AD15" t="s">
         <v>282</v>
@@ -8434,16 +8434,16 @@
         <v>385</v>
       </c>
       <c r="AM15" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AN15" t="s">
-        <v>370</v>
+        <v>448</v>
       </c>
       <c r="AO15">
-        <v>0.98092693557487454</v>
+        <v>0.99582230548799566</v>
       </c>
       <c r="AP15">
-        <v>349.67284779396647</v>
+        <v>76.591066053413869</v>
       </c>
       <c r="AR15" t="s">
         <v>282</v>
@@ -8470,16 +8470,16 @@
         <v>504</v>
       </c>
       <c r="BA15" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="BB15" t="s">
-        <v>591</v>
+        <v>366</v>
       </c>
       <c r="BC15">
-        <v>0.99637036284424008</v>
+        <v>0.98180592470173533</v>
       </c>
       <c r="BD15">
-        <v>66.543347855598327</v>
+        <v>333.55804713485287</v>
       </c>
     </row>
     <row r="16" spans="2:56">
@@ -8544,16 +8544,16 @@
         <v>295</v>
       </c>
       <c r="Y16" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="Z16" t="s">
         <v>354</v>
       </c>
       <c r="AA16">
-        <v>0.99852430677621173</v>
+        <v>0.99636728996375623</v>
       </c>
       <c r="AB16">
-        <v>27.054375769451152</v>
+        <v>66.599683997802714</v>
       </c>
       <c r="AD16" t="s">
         <v>282</v>
@@ -8580,16 +8580,16 @@
         <v>387</v>
       </c>
       <c r="AM16" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="AN16" t="s">
-        <v>356</v>
+        <v>450</v>
       </c>
       <c r="AO16">
-        <v>0.93717435218793788</v>
+        <v>0.99869874972548245</v>
       </c>
       <c r="AP16">
-        <v>1151.8035432211395</v>
+        <v>23.856255032822389</v>
       </c>
       <c r="AR16" t="s">
         <v>282</v>
@@ -8616,16 +8616,16 @@
         <v>506</v>
       </c>
       <c r="BA16" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="BB16" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="BC16">
-        <v>0.99234935324205875</v>
+        <v>0.99253849155603513</v>
       </c>
       <c r="BD16">
-        <v>140.26185722892211</v>
+        <v>136.79432147269009</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -8690,16 +8690,16 @@
         <v>297</v>
       </c>
       <c r="Y17" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="Z17" t="s">
         <v>355</v>
       </c>
       <c r="AA17">
-        <v>0.99838604658336239</v>
+        <v>0.99628076912917996</v>
       </c>
       <c r="AB17">
-        <v>29.589145971689483</v>
+        <v>68.185899298368355</v>
       </c>
       <c r="AD17" t="s">
         <v>282</v>
@@ -8726,16 +8726,16 @@
         <v>389</v>
       </c>
       <c r="AM17" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="AN17" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="AO17">
-        <v>0.96551955124232614</v>
+        <v>0.99841760060377538</v>
       </c>
       <c r="AP17">
-        <v>632.14156055735509</v>
+        <v>29.010655597451841</v>
       </c>
       <c r="AR17" t="s">
         <v>282</v>
@@ -8762,16 +8762,16 @@
         <v>508</v>
       </c>
       <c r="BA17" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="BB17" t="s">
-        <v>355</v>
+        <v>596</v>
       </c>
       <c r="BC17">
-        <v>0.99536692897647694</v>
+        <v>0.973232135644435</v>
       </c>
       <c r="BD17">
-        <v>84.939635431255269</v>
+        <v>490.74417985202501</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -8836,16 +8836,16 @@
         <v>299</v>
       </c>
       <c r="Y18" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="Z18" t="s">
         <v>356</v>
       </c>
       <c r="AA18">
-        <v>0.94069903208664407</v>
+        <v>0.9981032549815434</v>
       </c>
       <c r="AB18">
-        <v>1087.1844117448593</v>
+        <v>34.773658671704098</v>
       </c>
       <c r="AD18" t="s">
         <v>282</v>
@@ -8872,16 +8872,16 @@
         <v>391</v>
       </c>
       <c r="AM18" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="AN18" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="AO18">
-        <v>0.99693456929731861</v>
+        <v>0.99781438034778358</v>
       </c>
       <c r="AP18">
-        <v>56.199562882493169</v>
+        <v>40.069693623967019</v>
       </c>
       <c r="AR18" t="s">
         <v>282</v>
@@ -8908,16 +8908,16 @@
         <v>510</v>
       </c>
       <c r="BA18" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="BB18" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="BC18">
-        <v>0.88199812838352587</v>
+        <v>0.99637036284424008</v>
       </c>
       <c r="BD18">
-        <v>2163.367646302027</v>
+        <v>66.543347855598327</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -8982,16 +8982,16 @@
         <v>301</v>
       </c>
       <c r="Y19" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="Z19" t="s">
         <v>357</v>
       </c>
       <c r="AA19">
-        <v>0.99756610784588629</v>
+        <v>0.97633688849282452</v>
       </c>
       <c r="AB19">
-        <v>44.621356158751233</v>
+        <v>433.82371096488447</v>
       </c>
       <c r="AD19" t="s">
         <v>282</v>
@@ -9018,16 +9018,16 @@
         <v>393</v>
       </c>
       <c r="AM19" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="AN19" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="AO19">
-        <v>0.99750949182367343</v>
+        <v>0.99870022163576544</v>
       </c>
       <c r="AP19">
-        <v>45.659316565986806</v>
+        <v>23.829270010966344</v>
       </c>
       <c r="AR19" t="s">
         <v>282</v>
@@ -9054,16 +9054,16 @@
         <v>512</v>
       </c>
       <c r="BA19" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="BB19" t="s">
-        <v>352</v>
+        <v>600</v>
       </c>
       <c r="BC19">
-        <v>0.97902641975794957</v>
+        <v>0.99681267676383467</v>
       </c>
       <c r="BD19">
-        <v>384.51563777092457</v>
+        <v>58.434259329697142</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -9128,16 +9128,16 @@
         <v>303</v>
       </c>
       <c r="Y20" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Z20" t="s">
         <v>358</v>
       </c>
       <c r="AA20">
-        <v>0.9972084849335241</v>
+        <v>0.99798824264234642</v>
       </c>
       <c r="AB20">
-        <v>51.177776218725121</v>
+        <v>36.882218223648351</v>
       </c>
       <c r="AD20" t="s">
         <v>282</v>
@@ -9164,16 +9164,16 @@
         <v>395</v>
       </c>
       <c r="AM20" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="AN20" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="AO20">
-        <v>0.99804155179341392</v>
+        <v>0.99807466477127271</v>
       </c>
       <c r="AP20">
-        <v>35.904883787411507</v>
+        <v>35.297812526667357</v>
       </c>
       <c r="AR20" t="s">
         <v>282</v>
@@ -9200,16 +9200,16 @@
         <v>514</v>
       </c>
       <c r="BA20" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="BB20" t="s">
-        <v>356</v>
+        <v>602</v>
       </c>
       <c r="BC20">
-        <v>0.96140381292129873</v>
+        <v>0.99602290686668338</v>
       </c>
       <c r="BD20">
-        <v>707.59676310952364</v>
+        <v>72.91337411080552</v>
       </c>
     </row>
     <row r="21" spans="2:56">
@@ -9274,16 +9274,16 @@
         <v>305</v>
       </c>
       <c r="Y21" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="Z21" t="s">
         <v>359</v>
       </c>
       <c r="AA21">
-        <v>0.99809166649408687</v>
+        <v>0.99116451092312863</v>
       </c>
       <c r="AB21">
-        <v>34.986114275074357</v>
+        <v>161.98396640930775</v>
       </c>
       <c r="AD21" t="s">
         <v>282</v>
@@ -9310,16 +9310,16 @@
         <v>397</v>
       </c>
       <c r="AM21" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="AN21" t="s">
-        <v>457</v>
+        <v>376</v>
       </c>
       <c r="AO21">
-        <v>0.99508023417818925</v>
+        <v>0.99192535126433146</v>
       </c>
       <c r="AP21">
-        <v>90.195706733197795</v>
+        <v>148.0352268205892</v>
       </c>
       <c r="AR21" t="s">
         <v>282</v>
@@ -9346,16 +9346,16 @@
         <v>516</v>
       </c>
       <c r="BA21" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="BB21" t="s">
-        <v>356</v>
+        <v>604</v>
       </c>
       <c r="BC21">
-        <v>0.97591598065988894</v>
+        <v>0.98822137145239475</v>
       </c>
       <c r="BD21">
-        <v>441.54035456870389</v>
+        <v>215.94152337276336</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -9420,16 +9420,16 @@
         <v>307</v>
       </c>
       <c r="Y22" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="Z22" t="s">
         <v>360</v>
       </c>
       <c r="AA22">
-        <v>0.99850557699173803</v>
+        <v>0.99900168239190124</v>
       </c>
       <c r="AB22">
-        <v>27.397755151469518</v>
+        <v>18.302489481810518</v>
       </c>
       <c r="AD22" t="s">
         <v>282</v>
@@ -9456,16 +9456,16 @@
         <v>399</v>
       </c>
       <c r="AM22" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="AN22" t="s">
-        <v>459</v>
+        <v>366</v>
       </c>
       <c r="AO22">
-        <v>0.99940622505963084</v>
+        <v>0.98092693557487454</v>
       </c>
       <c r="AP22">
-        <v>10.885873906767051</v>
+        <v>349.67284779396647</v>
       </c>
       <c r="AR22" t="s">
         <v>282</v>
@@ -9492,16 +9492,16 @@
         <v>518</v>
       </c>
       <c r="BA22" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="BB22" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="BC22">
-        <v>0.99412039195829205</v>
+        <v>0.99662747375050009</v>
       </c>
       <c r="BD22">
-        <v>107.79281409797902</v>
+        <v>61.829647907498845</v>
       </c>
     </row>
     <row r="23" spans="2:56">
@@ -9566,16 +9566,16 @@
         <v>309</v>
       </c>
       <c r="Y23" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="Z23" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="AA23">
-        <v>0.99621285878087551</v>
+        <v>0.94069903208664407</v>
       </c>
       <c r="AB23">
-        <v>69.43092235061502</v>
+        <v>1087.1844117448593</v>
       </c>
       <c r="AD23" t="s">
         <v>282</v>
@@ -9602,16 +9602,16 @@
         <v>401</v>
       </c>
       <c r="AM23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="AN23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="AO23">
-        <v>0.99827635377245738</v>
+        <v>0.99013353407586135</v>
       </c>
       <c r="AP23">
-        <v>31.600180838280902</v>
+        <v>180.88520860920943</v>
       </c>
       <c r="AR23" t="s">
         <v>282</v>
@@ -9638,16 +9638,16 @@
         <v>520</v>
       </c>
       <c r="BA23" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="BB23" t="s">
-        <v>491</v>
+        <v>608</v>
       </c>
       <c r="BC23">
-        <v>0.98292548292671178</v>
+        <v>0.99284590877035406</v>
       </c>
       <c r="BD23">
-        <v>313.03281301028323</v>
+        <v>131.158339210175</v>
       </c>
     </row>
     <row r="24" spans="2:56">
@@ -9712,16 +9712,16 @@
         <v>311</v>
       </c>
       <c r="Y24" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="Z24" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AA24">
-        <v>0.9975431479552237</v>
+        <v>0.99756610784588629</v>
       </c>
       <c r="AB24">
-        <v>45.042287487565297</v>
+        <v>44.621356158751233</v>
       </c>
       <c r="AD24" t="s">
         <v>282</v>
@@ -9748,16 +9748,16 @@
         <v>403</v>
       </c>
       <c r="AM24" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AN24" t="s">
-        <v>370</v>
+        <v>464</v>
       </c>
       <c r="AO24">
-        <v>0.98949004263841422</v>
+        <v>0.99869589057011365</v>
       </c>
       <c r="AP24">
-        <v>192.68255162907312</v>
+        <v>23.908672881248773</v>
       </c>
       <c r="AR24" t="s">
         <v>282</v>
@@ -9784,16 +9784,16 @@
         <v>522</v>
       </c>
       <c r="BA24" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="BB24" t="s">
-        <v>353</v>
+        <v>610</v>
       </c>
       <c r="BC24">
-        <v>0.98355967005268352</v>
+        <v>0.97803702976044449</v>
       </c>
       <c r="BD24">
-        <v>301.40604903413595</v>
+        <v>402.65445439185123</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -9858,16 +9858,16 @@
         <v>313</v>
       </c>
       <c r="Y25" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="Z25" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AA25">
-        <v>0.99636728996375623</v>
+        <v>0.9972084849335241</v>
       </c>
       <c r="AB25">
-        <v>66.599683997802714</v>
+        <v>51.177776218725121</v>
       </c>
       <c r="AD25" t="s">
         <v>282</v>
@@ -9894,16 +9894,16 @@
         <v>405</v>
       </c>
       <c r="AM25" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="AN25" t="s">
-        <v>464</v>
+        <v>357</v>
       </c>
       <c r="AO25">
-        <v>0.99811838305018963</v>
+        <v>0.93717435218793788</v>
       </c>
       <c r="AP25">
-        <v>34.496310746523356</v>
+        <v>1151.8035432211395</v>
       </c>
       <c r="AR25" t="s">
         <v>282</v>
@@ -9930,16 +9930,16 @@
         <v>524</v>
       </c>
       <c r="BA25" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
       <c r="BB25" t="s">
-        <v>605</v>
+        <v>357</v>
       </c>
       <c r="BC25">
-        <v>0.9973402418125219</v>
+        <v>0.95957195194316591</v>
       </c>
       <c r="BD25">
-        <v>48.762233437098502</v>
+        <v>741.18088104195795</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -10004,16 +10004,16 @@
         <v>315</v>
       </c>
       <c r="Y26" t="s">
-        <v>278</v>
+        <v>260</v>
       </c>
       <c r="Z26" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AA26">
-        <v>0.99628076912917996</v>
+        <v>0.99391268208184824</v>
       </c>
       <c r="AB26">
-        <v>68.185899298368355</v>
+        <v>111.60082849944791</v>
       </c>
       <c r="AD26" t="s">
         <v>282</v>
@@ -10040,16 +10040,16 @@
         <v>407</v>
       </c>
       <c r="AM26" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AN26" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AO26">
-        <v>0.9985928182686985</v>
+        <v>0.96551955124232614</v>
       </c>
       <c r="AP26">
-        <v>25.798331740528162</v>
+        <v>632.14156055735509</v>
       </c>
       <c r="AR26" t="s">
         <v>282</v>
@@ -10076,16 +10076,16 @@
         <v>526</v>
       </c>
       <c r="BA26" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="BB26" t="s">
-        <v>356</v>
+        <v>613</v>
       </c>
       <c r="BC26">
-        <v>0.934538160869965</v>
+        <v>0.99603667376986049</v>
       </c>
       <c r="BD26">
-        <v>1200.1337173839754</v>
+        <v>72.660980885890424</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -10150,16 +10150,16 @@
         <v>317</v>
       </c>
       <c r="Y27" t="s">
-        <v>280</v>
+        <v>263</v>
       </c>
       <c r="Z27" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AA27">
-        <v>0.9981032549815434</v>
+        <v>0.99871218762601011</v>
       </c>
       <c r="AB27">
-        <v>34.773658671704098</v>
+        <v>23.609893523147914</v>
       </c>
       <c r="AD27" t="s">
         <v>282</v>
@@ -10186,16 +10186,16 @@
         <v>409</v>
       </c>
       <c r="AM27" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="AN27" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="AO27">
-        <v>0.99769811225811866</v>
+        <v>0.99693456929731861</v>
       </c>
       <c r="AP27">
-        <v>42.201275267825203</v>
+        <v>56.199562882493169</v>
       </c>
       <c r="AR27" t="s">
         <v>282</v>
@@ -10222,16 +10222,16 @@
         <v>528</v>
       </c>
       <c r="BA27" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
       <c r="BB27" t="s">
-        <v>356</v>
+        <v>615</v>
       </c>
       <c r="BC27">
-        <v>0.94616153753972931</v>
+        <v>0.99017867813273497</v>
       </c>
       <c r="BD27">
-        <v>987.03847843829612</v>
+        <v>180.05756756652616</v>
       </c>
     </row>
     <row r="28" spans="2:56">
@@ -10296,16 +10296,16 @@
         <v>319</v>
       </c>
       <c r="Y28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Z28" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AA28">
-        <v>0.99900168239190124</v>
+        <v>0.99856748800713691</v>
       </c>
       <c r="AB28">
-        <v>18.302489481810518</v>
+        <v>26.26271986915707</v>
       </c>
       <c r="AD28" t="s">
         <v>282</v>
@@ -10332,16 +10332,16 @@
         <v>411</v>
       </c>
       <c r="AM28" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="AN28" t="s">
-        <v>353</v>
+        <v>471</v>
       </c>
       <c r="AO28">
-        <v>0.98814178187791379</v>
+        <v>0.99682717865030179</v>
       </c>
       <c r="AP28">
-        <v>217.40066557158059</v>
+        <v>58.168391411134159</v>
       </c>
       <c r="AR28" t="s">
         <v>282</v>
@@ -10368,16 +10368,16 @@
         <v>530</v>
       </c>
       <c r="BA28" t="s">
-        <v>608</v>
+        <v>616</v>
       </c>
       <c r="BB28" t="s">
-        <v>356</v>
+        <v>617</v>
       </c>
       <c r="BC28">
-        <v>0.97218956380622079</v>
+        <v>0.99504061303190972</v>
       </c>
       <c r="BD28">
-        <v>509.85799688595205</v>
+        <v>90.922094414988095</v>
       </c>
     </row>
     <row r="29" spans="2:56">
@@ -10442,16 +10442,16 @@
         <v>321</v>
       </c>
       <c r="Y29" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="Z29" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AA29">
-        <v>0.9488788277802801</v>
+        <v>0.97905685820454003</v>
       </c>
       <c r="AB29">
-        <v>937.22149069486488</v>
+        <v>383.95759958343297</v>
       </c>
       <c r="AD29" t="s">
         <v>282</v>
@@ -10478,10 +10478,10 @@
         <v>413</v>
       </c>
       <c r="AM29" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="AN29" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="AO29">
         <v>0.99762356494824644</v>
@@ -10514,16 +10514,16 @@
         <v>532</v>
       </c>
       <c r="BA29" t="s">
-        <v>609</v>
+        <v>618</v>
       </c>
       <c r="BB29" t="s">
-        <v>610</v>
+        <v>619</v>
       </c>
       <c r="BC29">
-        <v>0.9924172440074055</v>
+        <v>0.98779966071713954</v>
       </c>
       <c r="BD29">
-        <v>139.01719319756617</v>
+        <v>223.67288685244134</v>
       </c>
     </row>
     <row r="30" spans="2:56">
@@ -10588,16 +10588,16 @@
         <v>323</v>
       </c>
       <c r="Y30" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="Z30" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AA30">
-        <v>0.9977500892185478</v>
+        <v>0.99726055556014181</v>
       </c>
       <c r="AB30">
-        <v>41.248364326622962</v>
+        <v>50.223148064066145</v>
       </c>
       <c r="AD30" t="s">
         <v>282</v>
@@ -10624,10 +10624,10 @@
         <v>415</v>
       </c>
       <c r="AM30" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="AN30" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="AO30">
         <v>0.99669176136177262</v>
@@ -10660,16 +10660,16 @@
         <v>534</v>
       </c>
       <c r="BA30" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="BB30" t="s">
-        <v>612</v>
+        <v>621</v>
       </c>
       <c r="BC30">
-        <v>0.99114508565756532</v>
+        <v>0.98841501119699848</v>
       </c>
       <c r="BD30">
-        <v>162.34009627796874</v>
+        <v>212.39146138836088</v>
       </c>
     </row>
     <row r="31" spans="2:56">
@@ -10734,16 +10734,16 @@
         <v>325</v>
       </c>
       <c r="Y31" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="Z31" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AA31">
-        <v>0.9982812149336332</v>
+        <v>0.99825665520226836</v>
       </c>
       <c r="AB31">
-        <v>31.51105955005805</v>
+        <v>31.96132129174655</v>
       </c>
       <c r="AD31" t="s">
         <v>282</v>
@@ -10770,16 +10770,16 @@
         <v>417</v>
       </c>
       <c r="AM31" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="AN31" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="AO31">
-        <v>0.99682717865030179</v>
+        <v>0.99827635377245738</v>
       </c>
       <c r="AP31">
-        <v>58.168391411134159</v>
+        <v>31.600180838280902</v>
       </c>
       <c r="AR31" t="s">
         <v>282</v>
@@ -10806,16 +10806,16 @@
         <v>536</v>
       </c>
       <c r="BA31" t="s">
-        <v>613</v>
+        <v>622</v>
       </c>
       <c r="BB31" t="s">
-        <v>614</v>
+        <v>596</v>
       </c>
       <c r="BC31">
-        <v>0.99561586640696276</v>
+        <v>0.93089405249526469</v>
       </c>
       <c r="BD31">
-        <v>80.375782539015233</v>
+        <v>1266.9423709201483</v>
       </c>
     </row>
     <row r="32" spans="2:56">
@@ -10880,16 +10880,16 @@
         <v>327</v>
       </c>
       <c r="Y32" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="Z32" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AA32">
-        <v>0.98833720780868572</v>
+        <v>0.99894650606645485</v>
       </c>
       <c r="AB32">
-        <v>213.8178568407609</v>
+        <v>19.314055448326833</v>
       </c>
       <c r="AD32" t="s">
         <v>282</v>
@@ -10916,16 +10916,16 @@
         <v>419</v>
       </c>
       <c r="AM32" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="AN32" t="s">
-        <v>477</v>
+        <v>366</v>
       </c>
       <c r="AO32">
-        <v>0.99841760060377538</v>
+        <v>0.98949004263841422</v>
       </c>
       <c r="AP32">
-        <v>29.010655597451841</v>
+        <v>192.68255162907312</v>
       </c>
       <c r="AR32" t="s">
         <v>282</v>
@@ -10952,16 +10952,16 @@
         <v>538</v>
       </c>
       <c r="BA32" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="BB32" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="BC32">
-        <v>0.99253849155603513</v>
+        <v>0.99302778580016682</v>
       </c>
       <c r="BD32">
-        <v>136.79432147269009</v>
+        <v>127.82392699694152</v>
       </c>
     </row>
     <row r="33" spans="2:56">
@@ -11026,16 +11026,16 @@
         <v>329</v>
       </c>
       <c r="Y33" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="Z33" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AA33">
-        <v>0.99391268208184824</v>
+        <v>0.98179245618315802</v>
       </c>
       <c r="AB33">
-        <v>111.60082849944791</v>
+        <v>333.80496997543548</v>
       </c>
       <c r="AD33" t="s">
         <v>282</v>
@@ -11062,16 +11062,16 @@
         <v>421</v>
       </c>
       <c r="AM33" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AN33" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="AO33">
-        <v>0.99781438034778358</v>
+        <v>0.99750949182367343</v>
       </c>
       <c r="AP33">
-        <v>40.069693623967019</v>
+        <v>45.659316565986806</v>
       </c>
       <c r="AR33" t="s">
         <v>282</v>
@@ -11098,16 +11098,16 @@
         <v>540</v>
       </c>
       <c r="BA33" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="BB33" t="s">
-        <v>618</v>
+        <v>357</v>
       </c>
       <c r="BC33">
-        <v>0.973232135644435</v>
+        <v>0.97591598065988894</v>
       </c>
       <c r="BD33">
-        <v>490.74417985202501</v>
+        <v>441.54035456870389</v>
       </c>
     </row>
     <row r="34" spans="2:56">
@@ -11172,16 +11172,16 @@
         <v>331</v>
       </c>
       <c r="Y34" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="Z34" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AA34">
-        <v>0.99871218762601011</v>
+        <v>0.99852430677621173</v>
       </c>
       <c r="AB34">
-        <v>23.609893523147914</v>
+        <v>27.054375769451152</v>
       </c>
       <c r="AD34" t="s">
         <v>282</v>
@@ -11208,16 +11208,16 @@
         <v>423</v>
       </c>
       <c r="AM34" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="AN34" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="AO34">
-        <v>0.99013353407586135</v>
+        <v>0.99811838305018963</v>
       </c>
       <c r="AP34">
-        <v>180.88520860920943</v>
+        <v>34.496310746523356</v>
       </c>
       <c r="AR34" t="s">
         <v>282</v>
@@ -11244,16 +11244,16 @@
         <v>542</v>
       </c>
       <c r="BA34" t="s">
-        <v>619</v>
+        <v>626</v>
       </c>
       <c r="BB34" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
       <c r="BC34">
-        <v>0.98779966071713954</v>
+        <v>0.99412039195829205</v>
       </c>
       <c r="BD34">
-        <v>223.67288685244134</v>
+        <v>107.79281409797902</v>
       </c>
     </row>
     <row r="35" spans="2:56">
@@ -11318,16 +11318,16 @@
         <v>333</v>
       </c>
       <c r="Y35" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="Z35" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="AA35">
-        <v>0.99856748800713691</v>
+        <v>0.99838604658336239</v>
       </c>
       <c r="AB35">
-        <v>26.26271986915707</v>
+        <v>29.589145971689483</v>
       </c>
       <c r="AD35" t="s">
         <v>282</v>
@@ -11354,16 +11354,16 @@
         <v>425</v>
       </c>
       <c r="AM35" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AN35" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="AO35">
-        <v>0.99869589057011365</v>
+        <v>0.9985928182686985</v>
       </c>
       <c r="AP35">
-        <v>23.908672881248773</v>
+        <v>25.798331740528162</v>
       </c>
       <c r="AR35" t="s">
         <v>282</v>
@@ -11390,16 +11390,16 @@
         <v>544</v>
       </c>
       <c r="BA35" t="s">
-        <v>621</v>
+        <v>628</v>
       </c>
       <c r="BB35" t="s">
-        <v>622</v>
+        <v>444</v>
       </c>
       <c r="BC35">
-        <v>0.98841501119699848</v>
+        <v>0.98292548292671178</v>
       </c>
       <c r="BD35">
-        <v>212.39146138836088</v>
+        <v>313.03281301028323</v>
       </c>
     </row>
     <row r="36" spans="2:56">
@@ -11464,16 +11464,16 @@
         <v>335</v>
       </c>
       <c r="Y36" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Z36" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="AA36">
-        <v>0.97905685820454003</v>
+        <v>0.9977500892185478</v>
       </c>
       <c r="AB36">
-        <v>383.95759958343297</v>
+        <v>41.248364326622962</v>
       </c>
       <c r="AD36" t="s">
         <v>282</v>
@@ -11500,16 +11500,16 @@
         <v>427</v>
       </c>
       <c r="AM36" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="AN36" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="AO36">
-        <v>0.99686124252542985</v>
+        <v>0.99769811225811866</v>
       </c>
       <c r="AP36">
-        <v>57.543887033786262</v>
+        <v>42.201275267825203</v>
       </c>
       <c r="AR36" t="s">
         <v>282</v>
@@ -11536,16 +11536,16 @@
         <v>546</v>
       </c>
       <c r="BA36" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="BB36" t="s">
-        <v>618</v>
+        <v>359</v>
       </c>
       <c r="BC36">
-        <v>0.93089405249526469</v>
+        <v>0.98355967005268352</v>
       </c>
       <c r="BD36">
-        <v>1266.9423709201483</v>
+        <v>301.40604903413595</v>
       </c>
     </row>
     <row r="37" spans="2:56">
@@ -11610,16 +11610,16 @@
         <v>337</v>
       </c>
       <c r="Y37" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="Z37" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="AA37">
-        <v>0.97633688849282452</v>
+        <v>0.9982812149336332</v>
       </c>
       <c r="AB37">
-        <v>433.82371096488447</v>
+        <v>31.51105955005805</v>
       </c>
       <c r="AD37" t="s">
         <v>282</v>
@@ -11646,16 +11646,16 @@
         <v>429</v>
       </c>
       <c r="AM37" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AN37" t="s">
-        <v>487</v>
+        <v>359</v>
       </c>
       <c r="AO37">
-        <v>0.99710631799330929</v>
+        <v>0.98814178187791379</v>
       </c>
       <c r="AP37">
-        <v>53.050836789329388</v>
+        <v>217.40066557158059</v>
       </c>
       <c r="AR37" t="s">
         <v>282</v>
@@ -11682,16 +11682,16 @@
         <v>548</v>
       </c>
       <c r="BA37" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="BB37" t="s">
-        <v>625</v>
+        <v>370</v>
       </c>
       <c r="BC37">
-        <v>0.99302778580016682</v>
+        <v>0.97902641975794957</v>
       </c>
       <c r="BD37">
-        <v>127.82392699694152</v>
+        <v>384.51563777092457</v>
       </c>
     </row>
     <row r="38" spans="2:56">
@@ -11756,16 +11756,16 @@
         <v>339</v>
       </c>
       <c r="Y38" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="Z38" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="AA38">
-        <v>0.99726055556014181</v>
+        <v>0.98833720780868572</v>
       </c>
       <c r="AB38">
-        <v>50.223148064066145</v>
+        <v>213.8178568407609</v>
       </c>
       <c r="AD38" t="s">
         <v>282</v>
@@ -11798,10 +11798,10 @@
         <v>489</v>
       </c>
       <c r="AO38">
-        <v>0.99550555557680764</v>
+        <v>0.99804155179341392</v>
       </c>
       <c r="AP38">
-        <v>82.398147758527074</v>
+        <v>35.904883787411507</v>
       </c>
       <c r="AR38" t="s">
         <v>282</v>
@@ -11828,16 +11828,16 @@
         <v>550</v>
       </c>
       <c r="BA38" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="BB38" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="BC38">
-        <v>0.99366677237144974</v>
+        <v>0.9973402418125219</v>
       </c>
       <c r="BD38">
-        <v>116.10917319008783</v>
+        <v>48.762233437098502</v>
       </c>
     </row>
     <row r="39" spans="2:56">
@@ -11905,7 +11905,7 @@
         <v>270</v>
       </c>
       <c r="Z39" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AA39">
         <v>0.96189283472138964</v>
@@ -11944,10 +11944,10 @@
         <v>491</v>
       </c>
       <c r="AO39">
-        <v>0.93896180472603763</v>
+        <v>0.99508023417818925</v>
       </c>
       <c r="AP39">
-        <v>1119.0335800226442</v>
+        <v>90.195706733197795</v>
       </c>
       <c r="AR39" t="s">
         <v>282</v>
@@ -11974,16 +11974,16 @@
         <v>552</v>
       </c>
       <c r="BA39" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="BB39" t="s">
-        <v>629</v>
+        <v>357</v>
       </c>
       <c r="BC39">
-        <v>0.9205295464439136</v>
+        <v>0.96140381292129873</v>
       </c>
       <c r="BD39">
-        <v>1456.9583151949184</v>
+        <v>707.59676310952364</v>
       </c>
     </row>
     <row r="40" spans="2:56">
@@ -12090,10 +12090,10 @@
         <v>493</v>
       </c>
       <c r="AO40">
-        <v>0.99870022163576544</v>
+        <v>0.99940622505963084</v>
       </c>
       <c r="AP40">
-        <v>23.829270010966344</v>
+        <v>10.885873906767051</v>
       </c>
       <c r="AR40" t="s">
         <v>282</v>
@@ -12120,16 +12120,16 @@
         <v>554</v>
       </c>
       <c r="BA40" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="BB40" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="BC40">
-        <v>0.99519319222421976</v>
+        <v>0.99234935324205875</v>
       </c>
       <c r="BD40">
-        <v>88.124809222638589</v>
+        <v>140.26185722892211</v>
       </c>
     </row>
     <row r="41" spans="2:56">
@@ -12236,10 +12236,10 @@
         <v>495</v>
       </c>
       <c r="AO41">
-        <v>0.99807466477127271</v>
+        <v>0.99686124252542985</v>
       </c>
       <c r="AP41">
-        <v>35.297812526667357</v>
+        <v>57.543887033786262</v>
       </c>
       <c r="AR41" t="s">
         <v>282</v>
@@ -12266,16 +12266,16 @@
         <v>556</v>
       </c>
       <c r="BA41" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="BB41" t="s">
-        <v>633</v>
+        <v>372</v>
       </c>
       <c r="BC41">
-        <v>0.98822137145239475</v>
+        <v>0.99536692897647694</v>
       </c>
       <c r="BD41">
-        <v>215.94152337276336</v>
+        <v>84.939635431255269</v>
       </c>
     </row>
     <row r="42" spans="2:56">
@@ -12304,16 +12304,16 @@
         <v>558</v>
       </c>
       <c r="BA42" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="BB42" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="BC42">
-        <v>0.99662747375050009</v>
+        <v>0.88199812838352587</v>
       </c>
       <c r="BD42">
-        <v>61.829647907498845</v>
+        <v>2163.367646302027</v>
       </c>
     </row>
     <row r="43" spans="2:56">
@@ -12342,16 +12342,16 @@
         <v>560</v>
       </c>
       <c r="BA43" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="BB43" t="s">
-        <v>637</v>
+        <v>359</v>
       </c>
       <c r="BC43">
-        <v>0.99284590877035406</v>
+        <v>0.98235584693125277</v>
       </c>
       <c r="BD43">
-        <v>131.158339210175</v>
+        <v>323.47613959369914</v>
       </c>
     </row>
     <row r="44" spans="2:56">
@@ -12380,16 +12380,16 @@
         <v>562</v>
       </c>
       <c r="BA44" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="BB44" t="s">
-        <v>639</v>
+        <v>357</v>
       </c>
       <c r="BC44">
-        <v>0.97803702976044449</v>
+        <v>0.934538160869965</v>
       </c>
       <c r="BD44">
-        <v>402.65445439185123</v>
+        <v>1200.1337173839754</v>
       </c>
     </row>
     <row r="45" spans="2:56">
@@ -12418,16 +12418,16 @@
         <v>564</v>
       </c>
       <c r="BA45" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="BB45" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="BC45">
-        <v>0.95957195194316591</v>
+        <v>0.94616153753972931</v>
       </c>
       <c r="BD45">
-        <v>741.18088104195795</v>
+        <v>987.03847843829612</v>
       </c>
     </row>
     <row r="46" spans="2:56">
@@ -12456,16 +12456,16 @@
         <v>566</v>
       </c>
       <c r="BA46" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="BB46" t="s">
-        <v>642</v>
+        <v>357</v>
       </c>
       <c r="BC46">
-        <v>0.99603667376986049</v>
+        <v>0.97218956380622079</v>
       </c>
       <c r="BD46">
-        <v>72.660980885890424</v>
+        <v>509.85799688595205</v>
       </c>
     </row>
     <row r="47" spans="2:56">
@@ -12500,10 +12500,10 @@
         <v>644</v>
       </c>
       <c r="BC47">
-        <v>0.99017867813273497</v>
+        <v>0.9924172440074055</v>
       </c>
       <c r="BD47">
-        <v>180.05756756652616</v>
+        <v>139.01719319756617</v>
       </c>
     </row>
     <row r="48" spans="2:56">
@@ -12538,10 +12538,10 @@
         <v>646</v>
       </c>
       <c r="BC48">
-        <v>0.99504061303190972</v>
+        <v>0.99114508565756532</v>
       </c>
       <c r="BD48">
-        <v>90.922094414988095</v>
+        <v>162.34009627796874</v>
       </c>
     </row>
     <row r="49" spans="44:56">
@@ -12576,10 +12576,10 @@
         <v>648</v>
       </c>
       <c r="BC49">
-        <v>0.99490784156958001</v>
+        <v>0.99561586640696276</v>
       </c>
       <c r="BD49">
-        <v>93.356237891033686</v>
+        <v>80.375782539015233</v>
       </c>
     </row>
     <row r="50" spans="44:56">
@@ -12614,10 +12614,10 @@
         <v>650</v>
       </c>
       <c r="BC50">
-        <v>0.99015836110796274</v>
+        <v>0.99366677237144974</v>
       </c>
       <c r="BD50">
-        <v>180.43004635401576</v>
+        <v>116.10917319008783</v>
       </c>
     </row>
     <row r="51" spans="44:56">
@@ -12652,10 +12652,10 @@
         <v>652</v>
       </c>
       <c r="BC51">
-        <v>0.99623532634854861</v>
+        <v>0.9205295464439136</v>
       </c>
       <c r="BD51">
-        <v>69.01901694327529</v>
+        <v>1456.9583151949184</v>
       </c>
     </row>
     <row r="52" spans="44:56">
@@ -12690,10 +12690,10 @@
         <v>654</v>
       </c>
       <c r="BC52">
-        <v>0.9966173923071765</v>
+        <v>0.99519319222421976</v>
       </c>
       <c r="BD52">
-        <v>62.014474368430825</v>
+        <v>88.124809222638589</v>
       </c>
     </row>
     <row r="53" spans="44:56">
@@ -12725,13 +12725,13 @@
         <v>655</v>
       </c>
       <c r="BB53" t="s">
-        <v>370</v>
+        <v>467</v>
       </c>
       <c r="BC53">
-        <v>0.98180592470173533</v>
+        <v>0.95726256957223688</v>
       </c>
       <c r="BD53">
-        <v>333.55804713485287</v>
+        <v>783.51955784232393</v>
       </c>
     </row>
     <row r="54" spans="44:56">
@@ -12763,13 +12763,13 @@
         <v>656</v>
       </c>
       <c r="BB54" t="s">
-        <v>353</v>
+        <v>444</v>
       </c>
       <c r="BC54">
-        <v>0.98235584693125277</v>
+        <v>0.9437657388784082</v>
       </c>
       <c r="BD54">
-        <v>323.47613959369914</v>
+        <v>1030.9614538958492</v>
       </c>
     </row>
   </sheetData>
@@ -12778,7 +12778,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08EC2A48-DF6B-4F64-8BA8-D2C460BD53E0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05E0B7D-888D-4E63-BC18-E33F9A764257}">
   <dimension ref="B9:Z54"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12890,7 +12890,7 @@
         <v>657</v>
       </c>
       <c r="K11" t="s">
-        <v>480</v>
+        <v>461</v>
       </c>
       <c r="L11">
         <v>6.1151684514715345</v>
@@ -12923,7 +12923,7 @@
         <v>719</v>
       </c>
       <c r="X11" t="s">
-        <v>606</v>
+        <v>640</v>
       </c>
       <c r="Y11">
         <v>32.783999999999999</v>
@@ -12958,7 +12958,7 @@
         <v>659</v>
       </c>
       <c r="K12" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="L12">
         <v>4.1221966299799098</v>
@@ -12991,7 +12991,7 @@
         <v>721</v>
       </c>
       <c r="X12" t="s">
-        <v>607</v>
+        <v>641</v>
       </c>
       <c r="Y12">
         <v>36.320999999999998</v>
@@ -13026,7 +13026,7 @@
         <v>661</v>
       </c>
       <c r="K13" t="s">
-        <v>490</v>
+        <v>443</v>
       </c>
       <c r="L13">
         <v>6.7028485191473308E-2</v>
@@ -13059,7 +13059,7 @@
         <v>723</v>
       </c>
       <c r="X13" t="s">
-        <v>608</v>
+        <v>642</v>
       </c>
       <c r="Y13">
         <v>43.956000000000003</v>
@@ -13094,7 +13094,7 @@
         <v>663</v>
       </c>
       <c r="K14" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
       <c r="L14">
         <v>1.3102559495532347</v>
@@ -13127,7 +13127,7 @@
         <v>725</v>
       </c>
       <c r="X14" t="s">
-        <v>599</v>
+        <v>625</v>
       </c>
       <c r="Y14">
         <v>62.099249999999998</v>
@@ -13162,7 +13162,7 @@
         <v>665</v>
       </c>
       <c r="K15" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="L15">
         <v>51.171736048895305</v>
@@ -13195,7 +13195,7 @@
         <v>727</v>
       </c>
       <c r="X15" t="s">
-        <v>584</v>
+        <v>655</v>
       </c>
       <c r="Y15">
         <v>0.38324999999999998</v>
@@ -13230,7 +13230,7 @@
         <v>667</v>
       </c>
       <c r="K16" t="s">
-        <v>476</v>
+        <v>451</v>
       </c>
       <c r="L16">
         <v>27.131882337818411</v>
@@ -13263,7 +13263,7 @@
         <v>729</v>
       </c>
       <c r="X16" t="s">
-        <v>640</v>
+        <v>611</v>
       </c>
       <c r="Y16">
         <v>56.725499999999997</v>
@@ -13298,7 +13298,7 @@
         <v>669</v>
       </c>
       <c r="K17" t="s">
-        <v>486</v>
+        <v>439</v>
       </c>
       <c r="L17">
         <v>8.7915989873091043</v>
@@ -13331,7 +13331,7 @@
         <v>731</v>
       </c>
       <c r="X17" t="s">
-        <v>598</v>
+        <v>633</v>
       </c>
       <c r="Y17">
         <v>58.03275</v>
@@ -13366,7 +13366,7 @@
         <v>671</v>
       </c>
       <c r="K18" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="L18">
         <v>26.915511431987859</v>
@@ -13399,7 +13399,7 @@
         <v>733</v>
       </c>
       <c r="X18" t="s">
-        <v>594</v>
+        <v>636</v>
       </c>
       <c r="Y18">
         <v>22.079249999999998</v>
@@ -13434,7 +13434,7 @@
         <v>673</v>
       </c>
       <c r="K19" t="s">
-        <v>463</v>
+        <v>481</v>
       </c>
       <c r="L19">
         <v>7.5025171344716721</v>
@@ -13467,7 +13467,7 @@
         <v>735</v>
       </c>
       <c r="X19" t="s">
-        <v>626</v>
+        <v>649</v>
       </c>
       <c r="Y19">
         <v>29.961749999999999</v>
@@ -13502,7 +13502,7 @@
         <v>675</v>
       </c>
       <c r="K20" t="s">
-        <v>482</v>
+        <v>463</v>
       </c>
       <c r="L20">
         <v>21.853336570084423</v>
@@ -13535,7 +13535,7 @@
         <v>737</v>
       </c>
       <c r="X20" t="s">
-        <v>634</v>
+        <v>605</v>
       </c>
       <c r="Y20">
         <v>28.478249999999999</v>
@@ -13570,7 +13570,7 @@
         <v>677</v>
       </c>
       <c r="K21" t="s">
-        <v>492</v>
+        <v>455</v>
       </c>
       <c r="L21">
         <v>40.036304639772588</v>
@@ -13603,7 +13603,7 @@
         <v>739</v>
       </c>
       <c r="X21" t="s">
-        <v>632</v>
+        <v>603</v>
       </c>
       <c r="Y21">
         <v>117.89700000000001</v>
@@ -13638,7 +13638,7 @@
         <v>679</v>
       </c>
       <c r="K22" t="s">
-        <v>458</v>
+        <v>492</v>
       </c>
       <c r="L22">
         <v>7.0903888161806279</v>
@@ -13671,7 +13671,7 @@
         <v>741</v>
       </c>
       <c r="X22" t="s">
-        <v>609</v>
+        <v>643</v>
       </c>
       <c r="Y22">
         <v>75.481499999999997</v>
@@ -13706,7 +13706,7 @@
         <v>681</v>
       </c>
       <c r="K23" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="L23">
         <v>16.970662525397827</v>
@@ -13739,7 +13739,7 @@
         <v>743</v>
       </c>
       <c r="X23" t="s">
-        <v>604</v>
+        <v>631</v>
       </c>
       <c r="Y23">
         <v>10.68975</v>
@@ -13774,7 +13774,7 @@
         <v>683</v>
       </c>
       <c r="K24" t="s">
-        <v>478</v>
+        <v>453</v>
       </c>
       <c r="L24">
         <v>2.5242004930684354</v>
@@ -13807,7 +13807,7 @@
         <v>745</v>
       </c>
       <c r="X24" t="s">
-        <v>615</v>
+        <v>593</v>
       </c>
       <c r="Y24">
         <v>82.607249999999993</v>
@@ -13842,7 +13842,7 @@
         <v>685</v>
       </c>
       <c r="K25" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="L25">
         <v>5.5071261071764246</v>
@@ -13875,7 +13875,7 @@
         <v>747</v>
       </c>
       <c r="X25" t="s">
-        <v>653</v>
+        <v>590</v>
       </c>
       <c r="Y25">
         <v>22.785</v>
@@ -13910,7 +13910,7 @@
         <v>687</v>
       </c>
       <c r="K26" t="s">
-        <v>452</v>
+        <v>479</v>
       </c>
       <c r="L26">
         <v>8.4886449615793467</v>
@@ -13943,7 +13943,7 @@
         <v>749</v>
       </c>
       <c r="X26" t="s">
-        <v>645</v>
+        <v>616</v>
       </c>
       <c r="Y26">
         <v>63.731250000000003</v>
@@ -13978,7 +13978,7 @@
         <v>689</v>
       </c>
       <c r="K27" t="s">
-        <v>454</v>
+        <v>488</v>
       </c>
       <c r="L27">
         <v>8.4075540995285696</v>
@@ -14011,7 +14011,7 @@
         <v>751</v>
       </c>
       <c r="X27" t="s">
-        <v>630</v>
+        <v>653</v>
       </c>
       <c r="Y27">
         <v>28.239750000000001</v>
@@ -14046,7 +14046,7 @@
         <v>691</v>
       </c>
       <c r="K28" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="L28">
         <v>15.703622047270191</v>
@@ -14079,7 +14079,7 @@
         <v>753</v>
       </c>
       <c r="X28" t="s">
-        <v>655</v>
+        <v>592</v>
       </c>
       <c r="Y28">
         <v>38.15925</v>
@@ -14114,7 +14114,7 @@
         <v>693</v>
       </c>
       <c r="K29" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="L29">
         <v>24.074478129461852</v>
@@ -14147,7 +14147,7 @@
         <v>755</v>
       </c>
       <c r="X29" t="s">
-        <v>597</v>
+        <v>630</v>
       </c>
       <c r="Y29">
         <v>3.38625</v>
@@ -14182,7 +14182,7 @@
         <v>695</v>
       </c>
       <c r="K30" t="s">
-        <v>456</v>
+        <v>490</v>
       </c>
       <c r="L30">
         <v>12.527007796473459</v>
@@ -14215,7 +14215,7 @@
         <v>757</v>
       </c>
       <c r="X30" t="s">
-        <v>638</v>
+        <v>609</v>
       </c>
       <c r="Y30">
         <v>30.597750000000001</v>
@@ -14250,7 +14250,7 @@
         <v>697</v>
       </c>
       <c r="K31" t="s">
-        <v>494</v>
+        <v>457</v>
       </c>
       <c r="L31">
         <v>22.322239264526591</v>
@@ -14283,7 +14283,7 @@
         <v>759</v>
       </c>
       <c r="X31" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="Y31">
         <v>98.024249999999995</v>
@@ -14318,7 +14318,7 @@
         <v>699</v>
       </c>
       <c r="K32" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="L32">
         <v>13.047413180463023</v>
@@ -14351,7 +14351,7 @@
         <v>761</v>
       </c>
       <c r="X32" t="s">
-        <v>603</v>
+        <v>629</v>
       </c>
       <c r="Y32">
         <v>28.459499999999998</v>
@@ -14386,7 +14386,7 @@
         <v>701</v>
       </c>
       <c r="K33" t="s">
-        <v>450</v>
+        <v>468</v>
       </c>
       <c r="L33">
         <v>23.637816650626842</v>
@@ -14419,7 +14419,7 @@
         <v>763</v>
       </c>
       <c r="X33" t="s">
-        <v>656</v>
+        <v>639</v>
       </c>
       <c r="Y33">
         <v>33.609749999999998</v>
@@ -14454,7 +14454,7 @@
         <v>703</v>
       </c>
       <c r="K34" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="L34">
         <v>50.076680799526407</v>
@@ -14487,7 +14487,7 @@
         <v>765</v>
       </c>
       <c r="X34" t="s">
-        <v>649</v>
+        <v>586</v>
       </c>
       <c r="Y34">
         <v>58.474499999999999</v>
@@ -14522,7 +14522,7 @@
         <v>705</v>
       </c>
       <c r="K35" t="s">
-        <v>467</v>
+        <v>485</v>
       </c>
       <c r="L35">
         <v>48.700042766740395</v>
@@ -14555,7 +14555,7 @@
         <v>767</v>
       </c>
       <c r="X35" t="s">
-        <v>613</v>
+        <v>647</v>
       </c>
       <c r="Y35">
         <v>18.711749999999999</v>
@@ -14590,7 +14590,7 @@
         <v>707</v>
       </c>
       <c r="K36" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="L36">
         <v>10.552785706661558</v>
@@ -14623,7 +14623,7 @@
         <v>769</v>
       </c>
       <c r="X36" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="Y36">
         <v>29.186250000000001</v>
@@ -14658,7 +14658,7 @@
         <v>709</v>
       </c>
       <c r="K37" t="s">
-        <v>488</v>
+        <v>441</v>
       </c>
       <c r="L37">
         <v>39.022668784713879</v>
@@ -14691,7 +14691,7 @@
         <v>771</v>
       </c>
       <c r="X37" t="s">
-        <v>611</v>
+        <v>645</v>
       </c>
       <c r="Y37">
         <v>14.49</v>
@@ -14726,7 +14726,7 @@
         <v>711</v>
       </c>
       <c r="K38" t="s">
-        <v>445</v>
+        <v>459</v>
       </c>
       <c r="L38">
         <v>33.851015501811965</v>
@@ -14759,7 +14759,7 @@
         <v>773</v>
       </c>
       <c r="X38" t="s">
-        <v>592</v>
+        <v>634</v>
       </c>
       <c r="Y38">
         <v>64.437749999999994</v>
@@ -14794,7 +14794,7 @@
         <v>713</v>
       </c>
       <c r="K39" t="s">
-        <v>462</v>
+        <v>478</v>
       </c>
       <c r="L39">
         <v>29.76120824924126</v>
@@ -14827,7 +14827,7 @@
         <v>775</v>
       </c>
       <c r="X39" t="s">
-        <v>647</v>
+        <v>584</v>
       </c>
       <c r="Y39">
         <v>59.085000000000001</v>
@@ -14862,7 +14862,7 @@
         <v>715</v>
       </c>
       <c r="K40" t="s">
-        <v>469</v>
+        <v>487</v>
       </c>
       <c r="L40">
         <v>26.081770464705624</v>
@@ -14895,7 +14895,7 @@
         <v>777</v>
       </c>
       <c r="X40" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="Y40">
         <v>37.460250000000002</v>
@@ -14930,7 +14930,7 @@
         <v>717</v>
       </c>
       <c r="K41" t="s">
-        <v>446</v>
+        <v>460</v>
       </c>
       <c r="L41">
         <v>28.326303899090867</v>
@@ -14963,7 +14963,7 @@
         <v>779</v>
       </c>
       <c r="X41" t="s">
-        <v>641</v>
+        <v>612</v>
       </c>
       <c r="Y41">
         <v>27.642749999999999</v>
@@ -14998,7 +14998,7 @@
         <v>781</v>
       </c>
       <c r="X42" t="s">
-        <v>600</v>
+        <v>626</v>
       </c>
       <c r="Y42">
         <v>62.597250000000003</v>
@@ -15033,7 +15033,7 @@
         <v>783</v>
       </c>
       <c r="X43" t="s">
-        <v>585</v>
+        <v>656</v>
       </c>
       <c r="Y43">
         <v>17.07525</v>
@@ -15068,7 +15068,7 @@
         <v>785</v>
       </c>
       <c r="X44" t="s">
-        <v>595</v>
+        <v>637</v>
       </c>
       <c r="Y44">
         <v>0.42149999999999999</v>
@@ -15103,7 +15103,7 @@
         <v>787</v>
       </c>
       <c r="X45" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="Y45">
         <v>5.7389999999999999</v>
@@ -15138,7 +15138,7 @@
         <v>789</v>
       </c>
       <c r="X46" t="s">
-        <v>628</v>
+        <v>651</v>
       </c>
       <c r="Y46">
         <v>1.81725</v>
@@ -15173,7 +15173,7 @@
         <v>791</v>
       </c>
       <c r="X47" t="s">
-        <v>602</v>
+        <v>628</v>
       </c>
       <c r="Y47">
         <v>15.998250000000001</v>
@@ -15208,7 +15208,7 @@
         <v>793</v>
       </c>
       <c r="X48" t="s">
-        <v>617</v>
+        <v>595</v>
       </c>
       <c r="Y48">
         <v>6.5272500000000004</v>
@@ -15243,7 +15243,7 @@
         <v>795</v>
       </c>
       <c r="X49" t="s">
-        <v>643</v>
+        <v>614</v>
       </c>
       <c r="Y49">
         <v>42.144750000000002</v>
@@ -15278,7 +15278,7 @@
         <v>797</v>
       </c>
       <c r="X50" t="s">
-        <v>586</v>
+        <v>599</v>
       </c>
       <c r="Y50">
         <v>16.497</v>
@@ -15313,7 +15313,7 @@
         <v>799</v>
       </c>
       <c r="X51" t="s">
-        <v>636</v>
+        <v>607</v>
       </c>
       <c r="Y51">
         <v>33.036000000000001</v>
@@ -15348,7 +15348,7 @@
         <v>801</v>
       </c>
       <c r="X52" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="Y52">
         <v>31.234500000000001</v>
@@ -15383,7 +15383,7 @@
         <v>803</v>
       </c>
       <c r="X53" t="s">
-        <v>588</v>
+        <v>601</v>
       </c>
       <c r="Y53">
         <v>30.527249999999999</v>
@@ -15418,7 +15418,7 @@
         <v>805</v>
       </c>
       <c r="X54" t="s">
-        <v>651</v>
+        <v>588</v>
       </c>
       <c r="Y54">
         <v>17.390999999999998</v>
@@ -15433,7 +15433,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9C78ACE-F1AB-4BE3-9C46-9E0EBD4A5397}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AC73FD5-C733-48CB-967D-49F8EF5CB3FB}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -17250,7 +17250,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C58D07B2-C206-4ADA-8DFE-7A743EA0D1E9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9076CAE5-2016-4E48-81C6-DB8D7A193F34}">
   <dimension ref="B2:M13"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>